<commit_message>
feat: update excel structure for kardex processing
</commit_message>
<xml_diff>
--- a/templates/kardex_estructura.xlsx
+++ b/templates/kardex_estructura.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\Filtro_Kardex\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB63FDD3-07EB-467B-B930-D444C195D9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E75D7F28-84A4-4659-A632-E5E543C6139B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{6F4D1C03-D4A0-443A-84E8-9BFAA0EC31BD}"/>
   </bookViews>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
-  <si>
-    <t>Código</t>
-  </si>
-  <si>
-    <t>Descripción</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="18">
   <si>
     <t>COMPROBANTE</t>
   </si>
@@ -89,13 +83,13 @@
     <t>01 Venta</t>
   </si>
   <si>
-    <t>021117</t>
-  </si>
-  <si>
-    <t>BS07</t>
-  </si>
-  <si>
-    <t>Maiz blanco molido</t>
+    <t>CODIGO</t>
+  </si>
+  <si>
+    <t>011012</t>
+  </si>
+  <si>
+    <t>BS41</t>
   </si>
 </sst>
 </file>
@@ -109,7 +103,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +119,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -134,7 +134,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -146,43 +146,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -224,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,7 +195,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -250,25 +212,17 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -605,200 +559,561 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB6C7049-6D05-43E0-8A23-66C443100E50}">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="14" t="s">
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="G1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="16" t="s">
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="12"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="11" t="s">
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+    </row>
+    <row r="2" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="12"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="11" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="12"/>
-      <c r="P1" s="13"/>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3">
+        <v>45290</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9">
+        <v>0</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0</v>
+      </c>
+      <c r="M3" s="8">
+        <v>141.74299999999999</v>
+      </c>
+      <c r="N3" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O3" s="8">
+        <v>5206.6572226600001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3">
+        <v>45293</v>
+      </c>
+      <c r="C4" s="4">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50530</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>1</v>
+      </c>
+      <c r="K4" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L4" s="8">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="M4" s="8">
+        <v>140.74299999999999</v>
+      </c>
+      <c r="N4" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O4" s="8">
+        <v>5169.9241426600001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3">
+        <v>45293</v>
+      </c>
+      <c r="C5" s="4">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="6">
+        <v>50538</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="K5" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L5" s="8">
+        <v>18.366540000000001</v>
+      </c>
+      <c r="M5" s="8">
+        <v>140.24299999999999</v>
+      </c>
+      <c r="N5" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O5" s="8">
+        <v>5151.5576026600002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3">
+        <v>45293</v>
+      </c>
+      <c r="C6" s="4">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="6">
+        <v>505995</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>1.4039999999999999</v>
+      </c>
+      <c r="K6" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L6" s="8">
+        <v>51.573244000000003</v>
+      </c>
+      <c r="M6" s="8">
+        <v>138.839</v>
+      </c>
+      <c r="N6" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O6" s="8">
+        <v>5099.98435866</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3">
+        <v>45295</v>
+      </c>
+      <c r="C7" s="4">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="6">
+        <v>50728</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0</v>
+      </c>
+      <c r="J7" s="8">
         <v>10</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>13</v>
+      <c r="K7" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L7" s="8">
+        <v>367.33080000000001</v>
+      </c>
+      <c r="M7" s="8">
+        <v>128.839</v>
+      </c>
+      <c r="N7" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O7" s="8">
+        <v>4732.6535586600003</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3">
+        <v>45297</v>
+      </c>
+      <c r="C8" s="4">
+        <v>3</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="4">
-        <v>45656</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E8" s="6">
+        <v>50708</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8">
+        <v>0.26</v>
+      </c>
+      <c r="K8" s="9">
+        <v>36.733080999999999</v>
+      </c>
+      <c r="L8" s="8">
+        <v>9.5506010000000003</v>
+      </c>
+      <c r="M8" s="8">
+        <v>128.57900000000001</v>
+      </c>
+      <c r="N8" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O8" s="8">
+        <v>4723.1029576600004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3">
+        <v>45300</v>
+      </c>
+      <c r="C9" s="4">
+        <v>3</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="6">
+        <v>50789</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G9" s="8">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8">
+        <v>5</v>
+      </c>
+      <c r="K9" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L9" s="8">
+        <v>183.66540000000001</v>
+      </c>
+      <c r="M9" s="8">
+        <v>123.57899999999999</v>
+      </c>
+      <c r="N9" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O9" s="8">
+        <v>4539.4375576599996</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="3">
+        <v>45301</v>
+      </c>
+      <c r="C10" s="4">
+        <v>3</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="6">
+        <v>53820</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="9">
-        <v>0</v>
-      </c>
-      <c r="I3" s="10">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9">
-        <f>+H3*I3</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="9">
-        <v>0</v>
-      </c>
-      <c r="L3" s="10">
-        <v>0</v>
-      </c>
-      <c r="M3" s="9">
-        <v>0</v>
-      </c>
-      <c r="N3" s="9">
-        <v>248090.39799999999</v>
-      </c>
-      <c r="O3" s="10">
-        <v>1.04626</v>
-      </c>
-      <c r="P3" s="9">
-        <f>+N3*O3</f>
-        <v>259567.05981147996</v>
+      <c r="G10" s="8">
+        <v>0</v>
+      </c>
+      <c r="H10" s="9">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0</v>
+      </c>
+      <c r="J10" s="8">
+        <v>5</v>
+      </c>
+      <c r="K10" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L10" s="8">
+        <v>183.66540000000001</v>
+      </c>
+      <c r="M10" s="8">
+        <v>118.57899999999999</v>
+      </c>
+      <c r="N10" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O10" s="8">
+        <v>4355.7721576599997</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3">
+        <v>45301</v>
+      </c>
+      <c r="C11" s="4">
+        <v>3</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="4">
-        <v>45659</v>
-      </c>
-      <c r="D4" s="5">
-        <v>4</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="7">
-        <v>50600</v>
-      </c>
-      <c r="G4" s="8" t="s">
+      <c r="E11" s="6">
+        <v>50822</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8">
+        <v>0</v>
+      </c>
+      <c r="J11" s="8">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="K11" s="9">
+        <v>36.733085000000003</v>
+      </c>
+      <c r="L11" s="8">
+        <v>3.0121129999999998</v>
+      </c>
+      <c r="M11" s="8">
+        <v>118.497</v>
+      </c>
+      <c r="N11" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O11" s="8">
+        <v>4352.7600446599999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="9">
-        <v>0</v>
-      </c>
-      <c r="I4" s="10">
-        <v>0</v>
-      </c>
-      <c r="J4" s="9">
-        <f>+H4*I4</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="9">
-        <v>447.59500000000003</v>
-      </c>
-      <c r="L4" s="10">
-        <v>1.04626</v>
-      </c>
-      <c r="M4" s="9">
-        <f>+K4*L4</f>
-        <v>468.3007447</v>
-      </c>
-      <c r="N4" s="9">
-        <v>247642.80300000001</v>
-      </c>
-      <c r="O4" s="10">
-        <v>1.04626</v>
-      </c>
-      <c r="P4" s="9">
-        <f>+P3+J4-M4</f>
-        <v>259098.75906677995</v>
+      <c r="B12" s="3">
+        <v>45302</v>
+      </c>
+      <c r="C12" s="4">
+        <v>3</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="6">
+        <v>50897</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="8">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8">
+        <v>5</v>
+      </c>
+      <c r="K12" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="L12" s="8">
+        <v>183.66540000000001</v>
+      </c>
+      <c r="M12" s="8">
+        <v>113.497</v>
+      </c>
+      <c r="N12" s="9">
+        <v>36.733080000000001</v>
+      </c>
+      <c r="O12" s="8">
+        <v>4169.0946446600001</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="N1:P1"/>
+  <mergeCells count="6">
+    <mergeCell ref="M1:O1"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="J1:L1"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>